<commit_message>
added new data and tab Infografias
</commit_message>
<xml_diff>
--- a/data/Negociado_de_Policia/npprDS_relacion.xlsx
+++ b/data/Negociado_de_Policia/npprDS_relacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Negociado_de_Policia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{406D0D6A-105D-467C-AF49-CE31B1E804E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8705D6CA-0F73-4368-8FE5-8BAA7905DCC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9756" yWindow="2448" windowWidth="11424" windowHeight="9420" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9720" yWindow="1716" windowWidth="12132" windowHeight="9384" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2019" sheetId="1" r:id="rId1"/>
@@ -1651,10 +1651,10 @@
         <v>2</v>
       </c>
       <c r="B2" s="2">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="C2" s="2">
-        <v>88</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1662,10 +1662,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="2">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C3" s="2">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1673,10 +1673,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="2">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C4" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1684,10 +1684,10 @@
         <v>5</v>
       </c>
       <c r="B5" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" s="2">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1695,10 +1695,10 @@
         <v>6</v>
       </c>
       <c r="B6" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C6" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1706,10 +1706,10 @@
         <v>7</v>
       </c>
       <c r="B7" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="C7" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1717,10 +1717,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="2">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C8" s="2">
-        <v>113</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1728,10 +1728,10 @@
         <v>9</v>
       </c>
       <c r="B9" s="2">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2">
-        <v>69</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1739,10 +1739,10 @@
         <v>10</v>
       </c>
       <c r="B10" s="2">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C10" s="2">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1750,10 +1750,10 @@
         <v>11</v>
       </c>
       <c r="B11" s="2">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C11" s="2">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1761,7 +1761,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2">
         <v>21</v>
@@ -1772,10 +1772,10 @@
         <v>13</v>
       </c>
       <c r="B13" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C13" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1783,10 +1783,10 @@
         <v>14</v>
       </c>
       <c r="B14" s="2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" s="2">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>